<commit_message>
tableau: add map for male countries
</commit_message>
<xml_diff>
--- a/excel/transformed-hovawart-litters-lk.xlsx
+++ b/excel/transformed-hovawart-litters-lk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martamucha-balcerek/Desktop/analityk danych/hovawart-lk-analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martamucha-balcerek/Desktop/analityk danych/hovawart-lk-analysis/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B61755-CF23-7340-A3EB-F5E184E7156D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39EA87B-163C-564B-9986-C67A67A17EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37120" yWindow="1020" windowWidth="27840" windowHeight="15100" xr2:uid="{6A024038-69FC-1E4C-AF5C-7988B9C8D9BB}"/>
+    <workbookView xWindow="-37120" yWindow="1020" windowWidth="27840" windowHeight="15100" activeTab="1" xr2:uid="{6A024038-69FC-1E4C-AF5C-7988B9C8D9BB}"/>
   </bookViews>
   <sheets>
     <sheet name="suka-hodowlana" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="112">
   <si>
     <t>blond</t>
   </si>
@@ -353,6 +353,27 @@
   </si>
   <si>
     <t>miot</t>
+  </si>
+  <si>
+    <t>kraj pochodzenia</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>Finland</t>
+  </si>
+  <si>
+    <t>Czech Republic</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>France</t>
   </si>
 </sst>
 </file>
@@ -902,7 +923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02F9B89B-083A-C543-AD30-14CF4DA2B772}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
@@ -913,7 +934,7 @@
     <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>23</v>
       </c>
@@ -932,8 +953,11 @@
       <c r="F1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -946,8 +970,11 @@
       <c r="D2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -960,8 +987,11 @@
       <c r="D3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -974,8 +1004,11 @@
       <c r="D4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -994,8 +1027,11 @@
       <c r="F5" s="1">
         <v>39566</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1008,8 +1044,11 @@
       <c r="D6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1022,8 +1061,11 @@
       <c r="D7" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1036,8 +1078,11 @@
       <c r="D8" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1050,8 +1095,11 @@
       <c r="D9" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1064,8 +1112,11 @@
       <c r="D10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1078,8 +1129,11 @@
       <c r="D11" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1092,8 +1146,11 @@
       <c r="D12" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G12" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1106,8 +1163,11 @@
       <c r="D13" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G13" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1120,8 +1180,11 @@
       <c r="D14" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1134,8 +1197,11 @@
       <c r="D15" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G15" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1148,8 +1214,11 @@
       <c r="D16" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G16" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1162,8 +1231,11 @@
       <c r="D17" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1176,8 +1248,11 @@
       <c r="D18" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1190,8 +1265,11 @@
       <c r="D19" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1203,6 +1281,9 @@
       </c>
       <c r="D20" t="s">
         <v>24</v>
+      </c>
+      <c r="G20" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>